<commit_message>
Initial commit of grading app
</commit_message>
<xml_diff>
--- a/AI_Grading_Project/graded_results.xlsx
+++ b/AI_Grading_Project/graded_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,7 +439,22 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Points_Awarded</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Justification</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Reasoning_Summary</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Full_Reasoning</t>
         </is>
       </c>
     </row>
@@ -457,12 +472,44 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes an inverse relationship where fishers catching fish causes fish population to decrease and fishers' population also decreases over time (point B). However, it does not elaborate on the feedback loop by describing how these relationships influence each other over time (point C) nor does it establish the feedback consequences over time (point D).</t>
+          <t>Feedback Loop Points A B C</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish and describes their inverse population relationship, also mentioning population replacement over time, but it lacks a clear explanation of the feedback consequences over time. No external system elements beyond fishers and fish are mentioned.</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Feedback loop points A, B, and C awarded for connection and relationship description; point D not awarded due to lack of feedback consequences explanation. No system elements points awarded as no external systems or impacts are described.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "fish get caught by fishers to be eaten/sold." Award 1 point.
+B (1 point): The response describes the relationship between fish and fisher populations: "fish population decreases and... their population decreases." This shows an inverse relationship. Award 1 point.
+C (1 point): The response mentions that "both populations are replaced over time," implying some recovery or replacement, which suggests a balancing loop. This is a different relationship connected to B. Award 1 point.
+D (1 point): The response does not clearly establish the feedback by explaining consequences over time leading to long-term stability or collapse. The phrase "both populations are replaced over time" is vague and does not explain the feedback mechanism or consequences. No point awarded.
+Step 2: System Elements Points
+E (1 point): The response does not mention any system elements beyond fishers and fish. No point awarded.
+F (1 point): Since E is not awarded, F cannot be awarded.
+Final points:
+Feedback Loop: 3/4
+System Elements: 0/2
+Total: 3/6
+{
+  "score": "3/6",
+  "points_awarded": "Feedback Loop Points A B C",
+  "justification": "The response clearly connects fishers and fish and describes their inverse population relationship, also mentioning population replacement over time, but it lacks a clear explanation of the feedback consequences over time. No external system elements beyond fishers and fish are mentioned.",
+  "reasoning_summary": "Feedback loop points A, B, and C awarded for connection and relationship description; point D not awarded due to lack of feedback consequences explanation. No system elements points awarded as no external systems or impacts are described."
+}</t>
         </is>
       </c>
     </row>
@@ -481,12 +528,41 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>4/4; 1/2</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>The response clearly indicates a connection between fishers and fish (A) and describes the inverse relationship between fish and fisher populations (B). It also establishes a balancing loop feedback by explaining how fishing restrictions allow fish populations to replenish (C and D). For systems elements, the response mentions financial costs influencing fishing behavior, which suggests an external system element (E), but it does not elaborate on broader system impacts (no point F).</t>
+          <t>A B C D E F</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>The response explicitly connects fishers and fish populations, describes their inverse relationship, explains balancing mechanisms like no-fishing periods and financial costs, and establishes the feedback loop consequences over time. It also mentions economic and regulatory system elements and their impact on the fish/fisher relationship.</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Feedback loop points A-D are earned sequentially by describing the connection, relationship, balancing mechanisms, and long-term consequences. System elements points E-F are earned by mentioning economic and regulatory factors and their impact on the fish/fisher system.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response states "The fishers fish; the population reduces over the season," indicating a connection between fishers and fish. Point A earned.
+B (1 point): The response describes the relationship: fish population reduces as fishers fish, and fishers sometimes stop fishing when it becomes too expensive. This shows an inverse relationship between fishers' activity and fish population. Point B earned.
+C (1 point): The response describes a balancing mechanism: "Then comes the period where the fishers aren't allowed to fish, allowing the fish population to replenish," and also "it gets too financially expensive to fish... which would sometimes make them stop fishing." This implies a balancing loop with regulatory or economic constraints limiting fishing. Point C earned.
+D (1 point): The response explains consequences over time leading to long-term stability: fish population replenishes during no-fishing periods, and financial cost limits overfishing. This establishes the feedback loop as balancing with consequences over time. Point D earned.
+Step 2: System Elements Points
+E (1 point): The response mentions economic factors ("too financially expensive to fish") and regulatory periods ("period where the fishers aren't allowed to fish"), which are system elements beyond fishers and fish. Point E earned.
+F (1 point): The response describes the impact of these system elements on the fish/fisher relationship: the no-fishing period allows fish population to replenish, and financial cost influences fishing behavior. This shows impact of broader systems on the fish/fisher relationship. Point F earned.
+Final score: 6/6
+{
+  "score": "6/6",
+  "points_awarded": "A B C D E F",
+  "justification": "The response explicitly connects fishers and fish populations, describes their inverse relationship, explains balancing mechanisms like no-fishing periods and financial costs, and establishes the feedback loop consequences over time. It also mentions economic and regulatory system elements and their impact on the fish/fisher relationship.",
+  "reasoning_summary": "Feedback loop points A-D are earned sequentially by describing the connection, relationship, balancing mechanisms, and long-term consequences. System elements points E-F are earned by mentioning economic and regulatory factors and their impact on the fish/fisher system."
+}</t>
         </is>
       </c>
     </row>
@@ -504,12 +580,56 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes the relationship between fish and fisher populations by implying a limit on fishing based on fish population recovery (point B). However, it does not elaborate on the feedback loop by describing how changes in one population affect the other over time (point C) nor does it establish the feedback consequences over time (point D). No system elements or broader system impacts are mentioned.</t>
+          <t>Feedback Loop Points, System Elements Points</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish, describes their inverse relationship, and explains consequences of overfishing leading to ecosystem destruction, establishing a balancing feedback loop. It also mentions the ecosystem and economic impacts, showing broader system elements and their interaction with the fish/fisher relationship.</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Feedback Loop: The response sequentially addresses the connection, relationship, consequences, and feedback mechanism as a balancing loop. System Elements: The response includes ecosystem and economic elements and describes their impact on and from the fish/fisher relationship.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+Yes. The response states "The fish act as the limit of how much the fishers can get at once," indicating fishers catch fish.  
+Award 1 point.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+Yes. The response says "the population is tied to the recovery rate" and "fishers can only fish up to a certain amount," implying that fish population limits fisher catch. This shows an inverse relationship: fish limit fishers' catch.  
+Award 1 point.
+C (1 point): For balancing loop, does the response describe another relationship connected to B but different, implying consequences such as fewer fish leading to fewer fishers or regulations?  
+The response says "unless they destroy the ecosystem and their money maker," implying consequences of overfishing leading to ecosystem destruction. This suggests a balancing loop where overfishing reduces fish, which then limits fishers.  
+Award 1 point.
+D (1 point): For balancing loop, does the response establish the feedback by explaining consequences over time leading to long-term stability?  
+The response implies that overfishing would destroy the ecosystem and the fishers' source of income, which suggests a feedback that would limit fishing to sustainable levels to avoid destruction. However, it does not explicitly state the long-term stability or cycles. The phrase "unless they destroy" implies a warning but not a clear feedback loop leading to stability.  
+This is borderline, but the response does establish a feedback mechanism that overfishing leads to ecosystem destruction, which would limit fishers, implying a balancing feedback.  
+Award 1 point.
+Total for Feedback Loop: 4/4
+Step 2: System Elements Points (2 points total)
+E (1 point): Does the response include system elements outside fishers and fish?  
+The response mentions "ecosystem" and "money maker," implying economic system and ecosystem beyond just fishers and fish.  
+Award 1 point.
+F (1 point): Does the response describe the impact of the fish/fisher relationship on the broader system or vice versa?  
+The response says "unless they destroy the ecosystem and their money maker," indicating that overfishing impacts the ecosystem and the economic livelihood of fishers. This describes the impact of the fish/fisher relationship on the broader system.  
+Award 1 point.
+Total for System Elements: 2/2
+Final score: 6/6
+{
+  "score": "6/6",
+  "points_awarded": "Feedback Loop Points, System Elements Points",
+  "justification": "The response clearly connects fishers and fish, describes their inverse relationship, and explains consequences of overfishing leading to ecosystem destruction, establishing a balancing feedback loop. It also mentions the ecosystem and economic impacts, showing broader system elements and their interaction with the fish/fisher relationship.",
+  "reasoning_summary": "Feedback Loop: The response sequentially addresses the connection, relationship, consequences, and feedback mechanism as a balancing loop. System Elements: The response includes ecosystem and economic elements and describes their impact on and from the fish/fisher relationship."
+}</t>
         </is>
       </c>
     </row>
@@ -527,12 +647,44 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes the relationship between fish and fisher populations by noting increased fishing due to technological advancements and population growth (point B). However, it does not clearly establish the feedback loop relationship (points C and D) or specify whether it is balancing or reinforcing. For systems points, it mentions economic impact beyond fishers and fish (point E) but does not describe the impact on the broader system (point F).</t>
+          <t>Feedback Loop Points A B, System Elements Points E</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>The response identifies the connection between fishers and fish and describes how fishing has increased due to technology and population growth, earning points A and B. It mentions broader system elements like the economy and environment, earning point E. However, it lacks a clear description of the feedback loop consequences and the impact of the fish/fisher relationship on the broader system, so points C, D, and F are not awarded.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Feedback Loop: Connection and relationship described but no feedback consequences explained. System Elements: External systems mentioned but no impact described.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish by mentioning "the act of fishing" and "Fisherman make a living off fishing." This satisfies point A.
+B (1 point): The response describes the relationship between fish and fisher populations by noting that "back then due to less technological advancements as well as a lower population the act of fishing was less, now due to advancements this act is much more common." This implies that more fishers or more fishing effort now exist due to technology and population changes, which affects fish. This satisfies point B.
+C (1 point): The response does not clearly describe another relationship connected to the feedback loop, such as consequences of fewer fish leading to fewer fishers or regulations, or for reinforcing loops, increased effort maintaining catch despite fewer fish. The mention of "many effects ranging across climate, the environment and the economy" is too vague and does not specify a feedback relationship. Therefore, point C is not awarded.
+D (1 point): Since point C is not awarded, point D cannot be awarded.
+Step 2: System Elements Points
+E (1 point): The response mentions "effects ranging across climate, the environment and the economy" and "Fisherman make a living off fishing and so do many middle men so the economy is very effected." This indicates system elements beyond fishers and fish, such as the economy and environment. This satisfies point E.
+F (1 point): The response does not describe the impact of the fish/fisher relationship on the broader system or vice versa in detail. It only states that the economy is "very effected" but does not explain how or the nature of the impact. Therefore, point F is not awarded.
+Final scoring:
+Feedback Loop Points: 2/4 (A and B)
+System Elements Points: 1/2 (E)
+Total: 3/6
+{
+  "score": "3/6",
+  "points_awarded": "Feedback Loop Points A B, System Elements Points E",
+  "justification": "The response identifies the connection between fishers and fish and describes how fishing has increased due to technology and population growth, earning points A and B. It mentions broader system elements like the economy and environment, earning point E. However, it lacks a clear description of the feedback loop consequences and the impact of the fish/fisher relationship on the broader system, so points C, D, and F are not awarded.",
+  "reasoning_summary": "Feedback Loop: Connection and relationship described but no feedback consequences explained. System Elements: External systems mentioned but no impact described."
+}</t>
         </is>
       </c>
     </row>
@@ -555,7 +707,36 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>The response clearly indicates the connection between fishers and fish (A), describes the inverse relationship between fish and fisher populations (B), elaborates on the balancing feedback loop with consequences and management interventions (C and D). It also includes system elements outside fishers and fish such as environmental changes, economic pressures, and policy interventions (E), and describes their impact on the fish/fisher relationship (F). Thus, it meets all criteria for full points in both feedback loop and systems elements.</t>
+          <t>Feedback Loop Points, System Elements Points</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>The response clearly identifies the feedback loop between fishers and fish populations, describing it as a balancing loop with consequences over time including management and technological innovation. It also mentions external system elements like environmental changes and policy interventions and explains their impact on the fish/fisher relationship.</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Criterion 1: The response sequentially addresses the feedback loop with clear relationships and long-term balancing consequences. Criterion 2: The response includes external system elements and describes their impact on the fish/fisher system.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Criterion 1: Feedback Loop Points  
+A (1 point): The response indicates a connection between fishers and fish ("fish populations grow, they attract more fishers," "overfishing can lead to a decline in fish populations").  
+B (1 point): The response describes the relationship between fish and fishers, explaining how fish populations and fishing efforts change relative to each other ("As fish populations grow, they attract more fishers," "overfishing can lead to a decline in fish populations, reducing catches and forcing fishers to either fish less or innovate").  
+C (1 point): The response describes another relationship connected to the balancing loop, mentioning consequences such as "innovate through new technologies or regulations," and "conservation or management measures to allow recovery."  
+D (1 point): The response establishes the feedback by explaining consequences over time leading to long-term stability ("This feedback loop illustrates a balancing system," "Effective management is critical to maintaining equilibrium and preventing overexploitation").  
+Criterion 2: System Elements Points  
+E (1 point): The response includes system elements outside of fishers and fish, such as "environmental changes, economic pressures, and policy interventions."  
+F (1 point): The response describes the impact of the fish/fisher relationship on the broader system or vice versa ("which shape both fish populations and the actions of fishers," "Effective management is critical to maintaining equilibrium").  
+Final score: 6/6
+{
+  "score": "6/6",
+  "points_awarded": "Feedback Loop Points, System Elements Points",
+  "justification": "The response clearly identifies the feedback loop between fishers and fish populations, describing it as a balancing loop with consequences over time including management and technological innovation. It also mentions external system elements like environmental changes and policy interventions and explains their impact on the fish/fisher relationship.",
+  "reasoning_summary": "Criterion 1: The response sequentially addresses the feedback loop with clear relationships and long-term balancing consequences. Criterion 2: The response includes external system elements and describes their impact on the fish/fisher system."
+}</t>
         </is>
       </c>
     </row>
@@ -573,12 +754,56 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>5/6</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish through the mention of fishing technology making it easier to catch fish (point A). It also implies that increased fishing decreases fish population (point B). However, it does not describe the relationship between fish and fishers in terms of population changes or feedback loops (points C and D), nor does it mention any broader system elements or impacts (points E and F). Therefore, only points A and B are partially met, resulting in a low overall score.</t>
+          <t>A B C E F</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish and describes how fishing technology increases catch efficiency, reducing fish populations (A, B, C). It mentions ecosystem endangerment as a broader system impact (E, F). However, it does not fully establish the feedback loop consequences over time leading to fishery collapse or unsustainability (D).</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded for connection, relationship, and reinforcing loop elaboration but not for full feedback consequences. System elements points awarded for mentioning ecosystems and describing impact on them.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+Yes. The response states "Advance technology ... make it much easier to catch them," indicating fishers catch fish.  
+Award 1 point.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+Yes. The response says "this decreases the population of the fish," implying more fishing reduces fish population.  
+Award 1 point.
+C (1 point): For reinforcing loop, does the response elaborate on the direct relationship, highlighting changes that maintain catch despite fewer fish (e.g., increased effort or new technology)?  
+Yes. The response says "progression of fishing technology ... make it much easier to catch them," which implies increased effort or efficiency despite fish population decline.  
+Award 1 point.
+D (1 point): For reinforcing loop, does the response establish feedback by explaining consequences over time leading to unsustainable overfishing and fishery collapse?  
+The response says "this decreases the population of the fish which could endanger many ecosystems," which implies negative consequences over time but does not explicitly state unsustainable overfishing or fishery collapse. The phrase "could endanger many ecosystems" is a potential consequence but not a clear feedback loop explanation of fishery collapse or unsustainability.  
+No clear explanation of feedback loop consequences over time leading to collapse or unsustainability.  
+No point awarded.
+Total for Feedback Loop: 3/4
+Step 2: System Elements Points (2 points total)
+E (1 point): Does the response include system elements outside fishers and fish?  
+Yes. The response mentions "endanger many ecosystems," which is a system element beyond fishers and fish.  
+Award 1 point.
+F (1 point): Does the response describe the impact of the fish/fisher relationship on the broader system or vice versa?  
+The response says "this decreases the population of the fish which could endanger many ecosystems," describing the impact of fish/fisher relationship on ecosystems.  
+Award 1 point.
+Total for System Elements: 2/2
+Final score: 5/6
+{
+  "score": "5/6",
+  "points_awarded": "A B C E F",
+  "justification": "The response clearly connects fishers and fish and describes how fishing technology increases catch efficiency, reducing fish populations (A, B, C). It mentions ecosystem endangerment as a broader system impact (E, F). However, it does not fully establish the feedback loop consequences over time leading to fishery collapse or unsustainability (D).",
+  "reasoning_summary": "Feedback loop points awarded for connection, relationship, and reinforcing loop elaboration but not for full feedback consequences. System elements points awarded for mentioning ecosystems and describing impact on them."
+}</t>
         </is>
       </c>
     </row>
@@ -596,12 +821,53 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) by stating fishers rely on fish for meals and livelihood. However, it does not describe the relationship between fish and fisher populations (point B), nor does it establish any feedback loop (points C and D). For systems points, it mentions health risks from fish eating plastic and bacteria, which is an external system element (point E), but does not describe the impact of the fish/fisher relationship on the broader system (point F). Overall, only point A and point E are met, resulting in a total of 1 point for feedback and 1 point for systems, but since the rubric requires sequential awarding and the system points are separate, the total score is 1/6.</t>
+          <t>A E F</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish (A) but does not describe population dynamics or feedback loops (no B, C, D). It mentions environmental pollution as an external system element (E) and explains its negative impact on fishers through fish consumption (F).</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Feedback loop points: only the basic connection between fishers and fish is made. System elements points: external environmental factors are mentioned and their impact on fishers is described.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+Yes. The response states "Fishers rely on fish for their meals" and "they are dependent on fish," indicating a connection.  
+Award 1 point.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+No. The response does not describe how fish or fisher populations increase or decrease relative to each other, or any dynamic relationship. It only states fishers rely on fish for food.  
+No point.
+C (1 point): Does the response describe another relationship connected to B, implying consequences such as fewer fish leading to fewer fishers or increased effort?  
+Not applicable since B was not earned.
+D (1 point): Does the response establish the feedback by explaining consequences over time leading to long-term stability or collapse?  
+Not applicable.
+Feedback Loop Points awarded: 1/4
+Step 2: System Elements Points (2 points total)
+E (1 point): Does the response include system elements outside of fishers and fish?  
+Yes. The response mentions "fish eat plastic and other bacteria that may be present in the ocean," which refers to environmental pollution affecting fish and indirectly fishers. This is an external system element (environmental pollution).  
+Award 1 point.
+F (1 point): Does the response describe the impact of the fish/fisher relationship on the broader system or vice versa?  
+Yes. The response states that fish eating plastic and bacteria "can affect the human body negatively and can even cause deaths," describing the impact of environmental pollution on fishers via fish consumption.  
+Award 1 point.
+System Elements Points awarded: 2/2
+Final score: 3/6
+{
+  "score": "3/6",
+  "points_awarded": "A E F",
+  "justification": "The response clearly connects fishers and fish (A) but does not describe population dynamics or feedback loops (no B, C, D). It mentions environmental pollution as an external system element (E) and explains its negative impact on fishers through fish consumption (F).",
+  "reasoning_summary": "Feedback loop points: only the basic connection between fishers and fish is made. System elements points: external environmental factors are mentioned and their impact on fishers is described."
+}</t>
         </is>
       </c>
     </row>
@@ -619,12 +885,41 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes the inverse relationship between fish and fisher populations (point B). It also describes a balancing loop by mentioning government restrictions that affect fish populations (point C). However, it does not fully establish the feedback over time or explain the long-term consequences of the fish and fisher relationship (point D). No system elements points were addressed.</t>
+          <t>A B C D E F</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>The response explicitly connects fishers and fish populations, describes their inverse relationship, explains government restrictions as a balancing feedback mechanism, and discusses how these restrictions impact fish population fluctuations over time. It also mentions external system elements (government and wildlife agencies) and their impact on the fish/fisher relationship.</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded sequentially for describing the inverse relationship and regulatory balancing loop; system elements points awarded for mentioning government agencies and their impact on the system.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "when there are an abundant amount of fishers the fish population tends to drop." This shows fishers catch fish and affect fish population. Award 1 point.
+B (1 point): The response describes the relationship between fish and fishers: more fishers cause fish population to drop; restrictions help fish population rise. This shows an inverse relationship. Award 1 point.
+C (1 point): The response describes another relationship connected to B but different: "government and wildlife agencies put limits or restrictions on how many fish people are allowed to catch." This implies consequences such as fewer fish leading to fewer fishers or regulations limiting catch, consistent with a balancing loop. Award 1 point.
+D (1 point): The response establishes the feedback by explaining consequences over time leading to long-term stability: "restrictions can change over time, allowing the fish population to fluctuate over time." This implies a balancing feedback loop with regulation and population fluctuation. Award 1 point.
+Step 2: System Elements Points
+E (1 point): The response mentions "government and wildlife agencies," which are external system elements beyond fishers and fish. Award 1 point.
+F (1 point): The response describes the impact of the fish/fisher relationship on the broader system or vice versa by explaining that "restrictions can change over time," implying that governmental systems impact fish/fisher dynamics. Award 1 point.
+Final score: 6/6
+{
+  "score": "6/6",
+  "points_awarded": "A B C D E F",
+  "justification": "The response explicitly connects fishers and fish populations, describes their inverse relationship, explains government restrictions as a balancing feedback mechanism, and discusses how these restrictions impact fish population fluctuations over time. It also mentions external system elements (government and wildlife agencies) and their impact on the fish/fisher relationship.",
+  "reasoning_summary": "Feedback loop points awarded sequentially for describing the inverse relationship and regulatory balancing loop; system elements points awarded for mentioning government agencies and their impact on the system."
+}</t>
         </is>
       </c>
     </row>
@@ -642,12 +937,51 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1/6</t>
+          <t>3/6</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) by mentioning fishers catching fish and selling them for consumption. However, it does not describe the relationship between fish and fisher populations (point B), nor does it address any feedback loop (points C and D). The mention of fish waste used as fertilizer and plants growing that fish eat introduces a system element outside of fishers and fish (point E), but it lacks explanation of the impact of this relationship on the broader system (point F). Overall, the response earns 1 point for feedback (A) and 1 point for systems (E), totaling 2 points, but since the rubric requires sequential awarding and the system points are separate, the score is 1/6 for feedback and 1/2 for systems; combined, this is 2/8, but as per instructions, only feedback and systems points are counted separately. Given the instructions and typical scoring, the best concise score is 1/6 for feedback and systems combined, reflecting minimal fulfillment.</t>
+          <t>A E F</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish by stating fishers catch fish (A). It includes system elements beyond fishers and fish by mentioning fertilizer and plants (E), and describes the impact of the fish/fisher relationship on the broader system through nutrient cycling (F). However, it does not describe the dynamic relationship or feedback loop between fish and fishers (B, C, D).</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded only for connection between fishers and fish. System elements points awarded for mentioning fertilizer and plants and describing their impact. No points for feedback loop dynamics or feedback mechanism.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Step 1: Evaluate Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+Yes. The response states "The fishers would fish and get the fish," indicating fishers catch fish.  
+=&gt; Award 1 point.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+No. The response does not describe how fish or fisher populations increase or decrease relative to each other, or any dynamic relationship. It only states fishers catch fish and eat or sell them.  
+=&gt; No point.
+Since B is not awarded, C and D cannot be awarded.
+Step 2: Evaluate System Elements Points (2 points total)
+E (1 point): Does the response include system elements outside of fishers and fish?  
+Yes. The response mentions "poop which would be used as fertilizer somewhere in the system growing plants in which fish would then eat." This introduces plants and fertilizer as external system elements beyond fishers and fish.  
+=&gt; Award 1 point.
+F (1 point): Does the response describe the impact of the fish/fisher relationship on the broader system or vice versa?  
+The response implies a cycle: fishers catch fish, fish are eaten, waste becomes fertilizer, plants grow, fish eat plants. This describes an impact of the fish/fisher relationship on the broader system (nutrient cycling and plant growth affecting fish).  
+=&gt; Award 1 point.
+Step 3: Final scoring
+Feedback Loop Points: 1/4 (only A)  
+System Elements Points: 2/2 (E and F)  
+Total: 3/6
+{
+  "score": "3/6",
+  "points_awarded": "A E F",
+  "justification": "The response clearly connects fishers and fish by stating fishers catch fish (A). It includes system elements beyond fishers and fish by mentioning fertilizer and plants (E), and describes the impact of the fish/fisher relationship on the broader system through nutrient cycling (F). However, it does not describe the dynamic relationship or feedback loop between fish and fishers (B, C, D).",
+  "reasoning_summary": "Feedback loop points awarded only for connection between fishers and fish. System elements points awarded for mentioning fertilizer and plants and describing their impact. No points for feedback loop dynamics or feedback mechanism."
+}</t>
         </is>
       </c>
     </row>
@@ -665,12 +999,41 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes a relationship between fish and fisher populations, noting that more fish benefit fishers (point B). However, it does not clearly describe the feedback loop or the consequences over time (points C and D) needed to demonstrate a balancing or reinforcing loop.</t>
+          <t>A B C D E F</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>The response explicitly connects fishers and fish, describes their relationship, implies a balancing feedback loop with sustainable fishing, and mentions the ocean ecosystem as a broader system element with mutual impacts.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded sequentially for connection, relationship, balancing loop implication, and feedback consequences; system elements points awarded for mentioning the ocean ecosystem and describing mutual impacts.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "The fisher need the fish to sell them," and "the fishes need the fishers to take care of the ocean for them." This clearly shows a relationship. Award 1 point.
+B (1 point): The response describes the relationship between fish and fishers: "The more fish there are the more the fishers benefit," and implies that fishers depend on fish abundance. This satisfies the description of how one population changes relative to the other. Award 1 point.
+C (1 point): The response states "they have to take care of the ocean and be sure not to fish them all at once," which implies a balancing relationship where fishers regulate their fishing to avoid depletion. This is a different relationship connected to B, implying consequences such as fewer fish leading to fewer fishers or regulations. Award 1 point.
+D (1 point): The response implies a feedback loop leading to long-term stability: "they have to take care of the ocean and be sure not to fish them all at once," suggesting sustainable fishing practices to maintain fish populations over time. This establishes the feedback mechanism and its consequences over time. Award 1 point.
+Step 2: System Elements Points
+E (1 point): The response mentions "take care of the ocean," which is an ecosystem element beyond just fishers and fish. This counts as mentioning system elements outside fishers and fish. Award 1 point.
+F (1 point): The response states "the fishes need the fishers to take care of the ocean for them," implying the impact of fishers on the ocean ecosystem and thus the broader system impact on fish/fisher relationship. This describes the impact of the fish/fisher relationship on the broader system or vice versa. Award 1 point.
+Final score: 6/6
+{
+  "score": "6/6",
+  "points_awarded": "A B C D E F",
+  "justification": "The response explicitly connects fishers and fish, describes their relationship, implies a balancing feedback loop with sustainable fishing, and mentions the ocean ecosystem as a broader system element with mutual impacts.",
+  "reasoning_summary": "Feedback loop points awarded sequentially for connection, relationship, balancing loop implication, and feedback consequences; system elements points awarded for mentioning the ocean ecosystem and describing mutual impacts."
+}</t>
         </is>
       </c>
     </row>
@@ -688,12 +1051,57 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes a relationship between fish and fisher populations (point B) by mentioning population changes and adaptation. However, it lacks a clear explanation of the feedback loop dynamics (points C and D) such as how these relationships cause balancing or reinforcing feedback over time. For systems elements, the response does not explicitly mention broader system elements outside fishers and fish (point E) nor does it describe the impact on broader systems (point F). Thus, it earns points A and B for feedback but no further points for feedback or systems.</t>
+          <t>Feedback Loop Points A B C, System Elements Points E</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish and describes their population relationship, including how humans adapt fishing methods, earning points A, B, and C. However, it lacks explanation of long-term feedback consequences, so point D is not awarded. The mention of humans using fishing for food and entertainment implies broader system elements, earning point E, but no impact on these systems is described, so point F is not awarded.</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Feedback Loop: Connection and relationship described with adaptation, but no long-term feedback consequences explained. System Elements: External elements implied by human use for food and entertainment, but no impact described.</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Step 1: Evaluate Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+- The response states "fishers over time have evolved fish to either migrate locations or adapt to fishing" and "Humans ... use fishing for food and entertainment." This indicates a connection between fishers and fish.  
+=&gt; Award 1 point for A.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+- The response says "Populations have increased for fish and humans, and both sides adapted to the other changes" and "The feedback loop changes depending on how many fish are born/die/caught." This implies a relationship where fish population changes affect humans and vice versa.  
+=&gt; Award 1 point for B.
+C (1 point): For balancing loop, describes another relationship connected but different implying consequences (e.g., fewer fish leading to fewer fishers or regulations). For reinforcing loop, elaborates on direct relationship highlighting changes maintaining catch despite fewer fish.  
+- The response says "Humans have changed the way of fishing to get a better advantage which affects the feedback loop." This suggests humans increase effort or technology to maintain catch despite fish changes, consistent with a reinforcing loop.  
+=&gt; Award 1 point for C.
+D (1 point): Establishes feedback by explaining consequences over time leading to unsustainable overfishing and fishery collapse (reinforcing) or long-term stability (balancing).  
+- The response does not explicitly explain consequences over time such as collapse or stability. It mentions adaptation but no clear long-term consequence or feedback outcome.  
+=&gt; Do not award point D.
+Step 2: Evaluate System Elements Points (2 points total)
+E (1 point): Includes system elements outside fishers and fish (ecosystems, economic systems, governmental systems, etc.)  
+- The response mentions "Humans are at the top of the food chain" and "fishing for food and entertainment," which implies human consumption and possibly economic or social systems. However, it does not explicitly mention external systems like ecosystems, government, or environment. The mention of "entertainment" could be considered a broader system element (economic or social).  
+- This is borderline, but "entertainment" and "humans at the top of the food chain" imply broader systems beyond just fishers and fish.  
+=&gt; Award 1 point for E.
+F (1 point): Describes impact of fish/fisher relationship on broader system or vice versa.  
+- The response does not describe how the fish/fisher relationship impacts or is impacted by the broader system. It only states humans use fishing for food and entertainment and that humans have changed fishing methods. No explicit impact on broader systems is described.  
+=&gt; Do not award point F.
+Final points:  
+Feedback Loop: A=1, B=1, C=1, D=0 → 3/4  
+System Elements: E=1, F=0 → 1/2  
+Total: 4/6
+{
+  "score": "4/6",
+  "points_awarded": "Feedback Loop Points A B C, System Elements Points E",
+  "justification": "The response clearly connects fishers and fish and describes their population relationship, including how humans adapt fishing methods, earning points A, B, and C. However, it lacks explanation of long-term feedback consequences, so point D is not awarded. The mention of humans using fishing for food and entertainment implies broader system elements, earning point E, but no impact on these systems is described, so point F is not awarded.",
+  "reasoning_summary": "Feedback Loop: Connection and relationship described with adaptation, but no long-term feedback consequences explained. System Elements: External elements implied by human use for food and entertainment, but no impact described."
+}</t>
         </is>
       </c>
     </row>
@@ -716,7 +1124,38 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) by describing fishers trying to catch fish and fish trying to avoid fake bait. However, it does not describe the relationship between fish and fisher populations (point B), nor does it elaborate on feedback loops (points C and D) or include any system elements (points E and F).</t>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>The response shows a basic connection between fishers and fish by describing fishers trying to catch fish and fish avoiding fake bait, earning point A. However, it lacks any description of population changes or feedback loops, and does not mention any broader system elements.</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Feedback loop: only connection between fishers and fish is stated without population or feedback details. System elements: no mention of external systems or impacts.</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "fishers try to catch fish" and "fish try to eat food without eating fake/trapped bait." This satisfies point A.
+B (1 point): The response does not describe how fish or fisher populations change relative to each other (e.g., increase or decrease in fish or fishers). No mention of population changes or consequences. So no point B.
+Since B is not earned, points C and D cannot be awarded.
+Step 2: System Elements Points
+E (1 point): The response does not mention any system elements beyond fishers and fish. No mention of ecosystems, economic systems, or other connected systems.
+F (1 point): Not applicable since E is not earned.
+Final scoring:
+Feedback Loop Points: 1/4 (only A)
+System Elements Points: 0/2
+Total: 1/6
+{
+  "score": "1/6",
+  "points_awarded": "A",
+  "justification": "The response shows a basic connection between fishers and fish by describing fishers trying to catch fish and fish avoiding fake bait, earning point A. However, it lacks any description of population changes or feedback loops, and does not mention any broader system elements.",
+  "reasoning_summary": "Feedback loop: only connection between fishers and fish is stated without population or feedback details. System elements: no mention of external systems or impacts."
+}</t>
         </is>
       </c>
     </row>
@@ -739,7 +1178,50 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes a relationship between fish and fisher populations, implying a direct relationship (point B). However, it lacks elaboration on the feedback loop (point C) and does not establish the feedback over time (point D). Additionally, the response does not mention any system elements outside of fishers and fish (point E) nor describe broader system impacts (point F).</t>
+          <t>A B</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish and describes a mutual relationship between their populations, earning points A and B. However, it lacks elaboration on feedback mechanisms or consequences over time, and does not mention any system elements beyond fishers and fish.</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Feedback Loop: The response identifies a connection and mutual influence between fishers and fish but does not elaborate on feedback consequences or mechanisms. System Elements: No external system elements or impacts are mentioned.</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Step 1: Evaluate Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+Yes. The response states "Fish serve as food and merchandise for fishers" and "Fishers consume fish and exchange them for money and other resources." This clearly indicates a connection.  
+Award 1 point.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+The response says, "An increase in the fish population could probably result in the fisher population. Vise Versa." This implies a relationship where fish population changes affect fisher population and vice versa, though it is vague and lacks detail. However, it does describe a relationship of mutual influence.  
+Award 1 point.
+C (1 point): For balancing loop, does the response describe another relationship connected to B but different, implying consequences such as fewer fish leading to fewer fishers, regulations, or fish farming? For reinforcing loop, does it elaborate on the direct relationship, highlighting changes that maintain catch despite fewer fish?  
+No. The response does not describe any additional relationship or consequences beyond the mutual influence statement. There is no mention of regulations, consequences, or feedback mechanisms.  
+No point.
+D (1 point): Does the response establish the feedback by explaining consequences over time leading to long-term stability or unsustainability?  
+No. The response does not explain consequences over time or feedback mechanisms.  
+No point.
+Total for Feedback Loop: 2/4
+Step 2: Evaluate System Elements Points (2 points total)
+E (1 point): Does the response include system elements outside of fishers and fish?  
+No. The response only mentions fishers and fish, with no mention of ecosystems, economic systems beyond fishers, government, environment, or other connected systems.  
+No point.
+F (1 point): Does the response describe the impact of the fish/fisher relationship on the broader system or vice versa?  
+No. Since no external system elements are mentioned, no impact is described.  
+No point.
+Total for System Elements: 0/2
+Final score: 2/6
+{
+  "score": "2/6",
+  "points_awarded": "A B",
+  "justification": "The response clearly connects fishers and fish and describes a mutual relationship between their populations, earning points A and B. However, it lacks elaboration on feedback mechanisms or consequences over time, and does not mention any system elements beyond fishers and fish.",
+  "reasoning_summary": "Feedback Loop: The response identifies a connection and mutual influence between fishers and fish but does not elaborate on feedback consequences or mechanisms. System Elements: No external system elements or impacts are mentioned."
+}</t>
         </is>
       </c>
     </row>
@@ -757,12 +1239,41 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2/4</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes the relationship between fish and fisher populations as a feedback loop with alternating increases and decreases (point B). However, it lacks elaboration on the implications of this relationship (point C) and does not establish the feedback consequences over time (point D). No system elements (points E or F) are mentioned.</t>
+          <t>A B C D</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>The response clearly shows a connection and relationship between fishers and fish populations, describing a balancing feedback loop cycle. However, it does not mention any system elements beyond fishers and fish or describe broader system impacts.</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded sequentially for describing a balancing loop cycle; no system elements mentioned, so no points awarded for system elements.</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "More fish-more fisher-less fish-less fisher- more fish." This shows fishers depend on fish and fish population changes relative to fishers. Award 1 point.
+B (1 point): The response describes the relationship between fish and fisher populations, explaining how one population changes relative to the other: more fish leads to more fishers, fewer fish leads to fewer fishers. Award 1 point.
+C (1 point): The response implies a balancing loop by showing the cycle "more fish-more fisher-less fish-less fisher-more fish," indicating consequences such as fewer fish leading to fewer fishers. Award 1 point.
+D (1 point): The response establishes the feedback by explaining consequences over time leading to long-term stability: the cycle implies a balancing feedback loop with predator-prey style oscillations. Award 1 point.
+Step 2: System Elements Points
+E (1 point): The response does not mention any system elements outside of fishers and fish (no mention of ecosystems, economic systems, government, environment, etc.). No point.
+F (1 point): Since E is not awarded, F cannot be awarded.
+Final score: 4/6
+{
+  "score": "4/6",
+  "points_awarded": "A B C D",
+  "justification": "The response clearly shows a connection and relationship between fishers and fish populations, describing a balancing feedback loop cycle. However, it does not mention any system elements beyond fishers and fish or describe broader system impacts.",
+  "reasoning_summary": "Feedback loop points awarded sequentially for describing a balancing loop cycle; no system elements mentioned, so no points awarded for system elements."
+}</t>
         </is>
       </c>
     </row>
@@ -780,12 +1291,56 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2/6</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>The response indicates a connection between fishers and fish (point A) and describes the inverse relationship where overfishing reduces fish populations (point B). However, it does not elaborate on the feedback loop relationship between fish and fishers (point C) or establish the feedback over time (point D). The mention of government involvement and sea laws hints at system elements but lacks explicit connection or impact on the fish/fisher relationship, so no system points are awarded.</t>
+          <t>A B C E</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish and describes their inverse relationship due to overfishing (A, B). It mentions government involvement as a regulatory factor (C). It includes external system elements like governments and global warming (E) but does not explain the feedback consequences over time or the impacts of these systems on fishers and fish (no D or F).</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded for connection, relationship, and regulatory involvement but not for explaining long-term feedback consequences. System elements point awarded for mentioning external systems but not for describing their impacts.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points (4 points total)
+A (1 point): Does the response indicate a connection between fishers and fish?  
+Yes. The response states "Fish and fisherman have a direct impact on each other" and "fish populations have dwindled due to over fishing." This clearly indicates a connection.  
+=&gt; Award 1 point.
+B (1 point): Does the response describe the relationship between fish and fisher populations, explaining how one changes relative to the other?  
+Yes. The response says "fish populations have dwindled due to over fishing," implying more fishers or fishing reduces fish populations. This describes an inverse relationship.  
+=&gt; Award 1 point.
+C (1 point): For balancing loop, does the response describe another relationship connected to B but different, implying consequences such as fewer fish leading to fewer fishers, regulations, or fish farming? For reinforcing loop, does it elaborate on the direct relationship?  
+The response mentions "Governments have involved themselves; however, sea laws are very difficult on a global basis." This implies regulations exist but are difficult to enforce, which is a different relationship connected to the fish/fisher relationship.  
+=&gt; Award 1 point.
+D (1 point): Does the response establish the feedback by explaining consequences over time leading to long-term stability (balancing) or unsustainable overfishing and collapse (reinforcing)?  
+The response states "There are both positive and negative feedback loops," but does not explain the consequences over time for the fish/fisher relationship specifically. The mention of global warming as a positive feedback loop is unrelated to fish/fisher feedback. No explanation of long-term consequences of the fish/fisher feedback loop is given.  
+=&gt; No point awarded.
+Step 2: System Elements Points (2 points total)
+E (1 point): Does the response include system elements outside of fishers and fish?  
+Yes. The response mentions "Governments have involved themselves" and "sea laws are very difficult on a global basis," which are governmental systems. It also mentions "Global warming," which is an environmental system.  
+=&gt; Award 1 point.
+F (1 point): Does the response describe the impact of the fish/fisher relationship on the broader system or vice versa?  
+No. The response does not describe how the fish/fisher relationship impacts governments or global warming, or how these systems impact fish/fisher dynamics. It only mentions these elements without describing impacts.  
+=&gt; No point awarded.
+Final tally:  
+Feedback Loop: 3/4 (A, B, C)  
+System Elements: 1/2 (E)  
+Total: 4/6
+{
+  "score": "4/6",
+  "points_awarded": "A B C E",
+  "justification": "The response clearly connects fishers and fish and describes their inverse relationship due to overfishing (A, B). It mentions government involvement as a regulatory factor (C). It includes external system elements like governments and global warming (E) but does not explain the feedback consequences over time or the impacts of these systems on fishers and fish (no D or F).",
+  "reasoning_summary": "Feedback loop points awarded for connection, relationship, and regulatory involvement but not for explaining long-term feedback consequences. System elements point awarded for mentioning external systems but not for describing their impacts."
+}</t>
         </is>
       </c>
     </row>
@@ -806,9 +1361,20 @@
           <t>0/6</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>The student response is empty and does not address any of the rubric criteria for feedback loops or system elements.</t>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No gradable content provided.</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>All criteria: 0 points — response is blank or insufficient.</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Response was blank or fewer than 5 words.</t>
         </is>
       </c>
     </row>
@@ -826,12 +1392,41 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4/4; 2/2</t>
+          <t>6/6</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>The response clearly establishes point A by indicating the connection between fishers and fish. Point B is met by describing how fish populations decline when fishermen catch too many fish, showing an inverse relationship. Point C is addressed by explaining that fishermen may capture fewer fish or change methods as a result, indicating a balancing feedback. Point D is fulfilled by describing the cycle of fish population recovery and the importance of sustainable fishing, establishing the feedback loop over time. For systems points, the response mentions fishermen depend on fish for livelihood (point E) and implies the broader system impact by emphasizing the need to fish properly to maintain long-term health of both fish and fishermen (point F).</t>
+          <t>A B C D E F</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>The response explicitly connects fishers and fish, describes their inverse relationship, elaborates on changes in fishing methods and fish recovery, and explains the long-term balancing feedback loop. It also mentions livelihood as a system element and discusses the importance of sustainable fishing for long-term health, showing impact on broader systems.</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Feedback loop points awarded sequentially for connection, relationship, additional relationships, and long-term feedback; system elements points awarded for mentioning livelihood and describing sustainability impact.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "fishermen depend on fish for their livelihood," "fish populations decline when fishermen catch too many of them." Award 1 point.
+B (1 point): The response describes the relationship between fish and fisher populations: "fish populations decline when fishermen catch too many," "fishermen may capture fewer fish or alter their fishing methods." This shows an inverse relationship. Award 1 point.
+C (1 point): The response describes another relationship connected to B: "fishermen may capture fewer fish or alter their fishing methods and locations," and "the number of fish can increase again if humans allow them time to recover." This implies consequences such as fewer fish leading to fewer fishers or changes in fishing methods, and fish population recovery. Award 1 point.
+D (1 point): The response establishes the feedback by explaining consequences over time leading to long-term stability: "This cycle demonstrates why it's critical to fish properly in order to maintain the long-term health of both fish and fishermen." This indicates a balancing loop with long-term stability. Award 1 point.
+Step 2: System Elements Points
+E (1 point): The response mentions "fishermen depend on fish for their livelihood," which is a system element outside of just fishers and fish (economic system/livelihood). Award 1 point.
+F (1 point): The response describes the impact of the fish/fisher relationship on the broader system: "This cycle demonstrates why it's critical to fish properly in order to maintain the long-term health of both fish and fishermen." This shows the impact on the livelihood system and sustainability. Award 1 point.
+Final score: 6/6
+{
+  "score": "6/6",
+  "points_awarded": "A B C D E F",
+  "justification": "The response explicitly connects fishers and fish, describes their inverse relationship, elaborates on changes in fishing methods and fish recovery, and explains the long-term balancing feedback loop. It also mentions livelihood as a system element and discusses the importance of sustainable fishing for long-term health, showing impact on broader systems.",
+  "reasoning_summary": "Feedback loop points awarded sequentially for connection, relationship, additional relationships, and long-term feedback; system elements points awarded for mentioning livelihood and describing sustainability impact."
+}</t>
         </is>
       </c>
     </row>
@@ -849,12 +1444,43 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>3/4</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>The response clearly indicates a connection between fishers and fish (point A) and describes the inverse relationship between fish and fisher populations (point B). It also describes the balancing loop feedback by explaining that fewer fish lead to fewer fishers (point C). However, it does not fully establish the long-term feedback consequences over time or elaborate on the cycle's stability (point D). No system elements beyond fishers and fish are mentioned, so no system points are awarded.</t>
+          <t>Feedback Loop Points</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>The response clearly connects fishers and fish, describes their inverse relationship, and explains a balancing feedback loop where fewer fish lead to fewer fishers, indicating long-term stability. However, it does not mention any system elements beyond fishers and fish or their impacts.</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Feedback loop points earned sequentially by describing the balancing loop; no system elements mentioned or impacts described.</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "Fishers use fish as a way to make their living." This shows fishers depend on fish.
+B (1 point): The response describes the relationship between fish and fishers: "When there are more fishers, there will be fewer fish." This shows an inverse relationship.
+C (1 point): The response describes another relationship connected to B: "Then when the fish resources becoming exhausive, there will be fewer fishers in the market." This implies fewer fish lead to fewer fishers, indicating a balancing loop.
+D (1 point): The response establishes the feedback over time leading to long-term stability: "when the fish resources becoming exhausive, there will be fewer fishers in the market." This implies a feedback loop that reduces fishers as fish decline, stabilizing the system.
+All four points A-D are earned.
+Step 2: System Elements Points
+E (1 point): The response does not mention any system elements beyond fishers and fish. No mention of ecosystems, economic systems, government, or other connected systems.
+F (1 point): Not applicable since E is not earned.
+No points for system elements.
+Final score: 4/6
+{
+  "score": "4/6",
+  "points_awarded": "Feedback Loop Points",
+  "justification": "The response clearly connects fishers and fish, describes their inverse relationship, and explains a balancing feedback loop where fewer fish lead to fewer fishers, indicating long-term stability. However, it does not mention any system elements beyond fishers and fish or their impacts.",
+  "reasoning_summary": "Feedback loop points earned sequentially by describing the balancing loop; no system elements mentioned or impacts described."
+}</t>
         </is>
       </c>
     </row>
@@ -873,12 +1499,41 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>4/4</t>
+          <t>4/6</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>The response clearly indicates the connection between fishers and fish (A), describes the inverse relationship between fish and fisher populations (B), elaborates on the connected relationship showing how changes in one population affect the other (C), and establishes the feedback loop over time demonstrating the balancing nature of the system (D).</t>
+          <t>Feedback Loop Points</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>The response clearly describes the connection and relationships between fishers and fish populations, identifying a balancing feedback loop and explaining the cyclical consequences over time. However, it does not mention any system elements beyond fishers and fish or their impacts.</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Feedback Loop Points: The response sequentially describes the balancing feedback loop between fishers and fish populations. System Elements Points: No external system elements or impacts are mentioned.</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Step 1: Feedback Loop Points
+A (1 point): The response indicates a connection between fishers and fish: "the number of fish in a pool increases --&gt; the number of fishers increases --&gt; the number of fish decreases --&gt; the number of fishers decreases." This shows fishers catch fish and fish population affects fishers. Award 1 point.
+B (1 point): The response describes the relationship between fish and fishers, explaining how one population changes relative to the other: more fish leads to more fishers, more fishers lead to fewer fish, fewer fish lead to fewer fishers, and fewer fishers lead to more fish. This is a direct description of population changes. Award 1 point.
+C (1 point): The response describes another relationship connected to the balancing loop: the cycle of fish and fishers increasing and decreasing. This implies consequences such as fewer fish leading to fewer fishers, which is a different relationship connected to the first. Award 1 point.
+D (1 point): The response states "This is a balance feedback loop," and the described cycle implies long-term stability through predator-prey style oscillations. Although brief, it establishes the feedback by explaining consequences over time leading to stability. Award 1 point.
+Step 2: System Elements Points
+E (1 point): The response does not mention any system elements beyond fishers and fish (no mention of ecosystems, economic systems, government, environment, etc.). No point.
+F (1 point): Since E is not awarded, F cannot be awarded.
+Final score: 4/6
+{
+  "score": "4/6",
+  "points_awarded": "Feedback Loop Points",
+  "justification": "The response clearly describes the connection and relationships between fishers and fish populations, identifying a balancing feedback loop and explaining the cyclical consequences over time. However, it does not mention any system elements beyond fishers and fish or their impacts.",
+  "reasoning_summary": "Feedback Loop Points: The response sequentially describes the balancing feedback loop between fishers and fish populations. System Elements Points: No external system elements or impacts are mentioned."
+}</t>
         </is>
       </c>
     </row>

</xml_diff>